<commit_message>
Leetcode 121- best time to buy and sell stock
</commit_message>
<xml_diff>
--- a/Top300_LeetCode_DSA_Questions.xlsx
+++ b/Top300_LeetCode_DSA_Questions.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1410" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1411" uniqueCount="902">
   <si>
     <t>🚀 TOP 300 LeetCode DSA Questions — MNC &amp; Startup Interview Prep</t>
   </si>
@@ -3186,7 +3186,7 @@
     <xf numFmtId="0" fontId="12" fillId="61" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="260">
+  <cellXfs count="261">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3881,6 +3881,13 @@
     <xf numFmtId="0" fontId="9" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="61" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3954,11 +3961,7 @@
     <xf numFmtId="0" fontId="5" fillId="60" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="61" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4279,22 +4282,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="234" t="s">
+      <c r="A1" s="237" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="232" t="s">
+      <c r="A2" s="235" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="4" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -4654,13 +4657,13 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="235" t="s">
+      <c r="A26" s="238" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="233"/>
-      <c r="C26" s="233"/>
-      <c r="D26" s="233"/>
-      <c r="E26" s="233"/>
+      <c r="B26" s="236"/>
+      <c r="C26" s="236"/>
+      <c r="D26" s="236"/>
+      <c r="E26" s="236"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4687,22 +4690,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="245" t="s">
+      <c r="A1" s="248" t="s">
         <v>414</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>415</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="97" t="s">
@@ -5000,22 +5003,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="246" t="s">
+      <c r="A1" s="249" t="s">
         <v>458</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>459</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="110" t="s">
@@ -5517,22 +5520,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="250" t="s">
         <v>541</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>542</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="123" t="s">
@@ -6000,22 +6003,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="248" t="s">
+      <c r="A1" s="251" t="s">
         <v>618</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>619</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="134" t="s">
@@ -6636,22 +6639,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="249" t="s">
+      <c r="A1" s="252" t="s">
         <v>708</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>709</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="146" t="s">
@@ -6915,22 +6918,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="250" t="s">
+      <c r="A1" s="253" t="s">
         <v>749</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>750</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="157" t="s">
@@ -7177,22 +7180,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="254" t="s">
         <v>775</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>776</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="160" t="s">
@@ -7439,22 +7442,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="252" t="s">
+      <c r="A1" s="255" t="s">
         <v>792</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>793</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="166" t="s">
@@ -7616,22 +7619,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="253" t="s">
+      <c r="A1" s="256" t="s">
         <v>811</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>812</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="169" t="s">
@@ -7878,22 +7881,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="254" t="s">
+      <c r="A1" s="257" t="s">
         <v>846</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>847</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="180" t="s">
@@ -8055,22 +8058,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="237" t="s">
+      <c r="A1" s="240" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -8088,7 +8091,7 @@
       <c r="E3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="257" t="s">
+      <c r="F3" s="232" t="s">
         <v>900</v>
       </c>
     </row>
@@ -8105,10 +8108,10 @@
       <c r="D4" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="E4" s="259" t="s">
+      <c r="E4" s="234" t="s">
         <v>78</v>
       </c>
-      <c r="F4" s="258" t="s">
+      <c r="F4" s="233" t="s">
         <v>901</v>
       </c>
     </row>
@@ -8122,11 +8125,14 @@
       <c r="C5" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="260" t="s">
         <v>80</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>81</v>
+      </c>
+      <c r="F5" s="233" t="s">
+        <v>901</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8714,6 +8720,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E4" r:id="rId1"/>
+    <hyperlink ref="D5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8734,22 +8741,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="255" t="s">
+      <c r="A1" s="258" t="s">
         <v>860</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>861</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="190" t="s">
@@ -8843,22 +8850,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="256" t="s">
+      <c r="A1" s="259" t="s">
         <v>871</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>872</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="200" t="s">
@@ -9088,22 +9095,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="241" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>187</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
@@ -9486,22 +9493,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="239" t="s">
+      <c r="A1" s="242" t="s">
         <v>248</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>249</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
@@ -9731,22 +9738,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="243" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>272</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="41" t="s">
@@ -9942,22 +9949,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="241" t="s">
+      <c r="A1" s="244" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>289</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="53" t="s">
@@ -10170,22 +10177,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="242" t="s">
+      <c r="A1" s="245" t="s">
         <v>311</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>312</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="65" t="s">
@@ -10483,22 +10490,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="246" t="s">
         <v>350</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>351</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="77" t="s">
@@ -10660,22 +10667,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="244" t="s">
+      <c r="A1" s="247" t="s">
         <v>370</v>
       </c>
-      <c r="B1" s="233"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="239" t="s">
         <v>371</v>
       </c>
-      <c r="B2" s="233"/>
-      <c r="C2" s="233"/>
-      <c r="D2" s="233"/>
-      <c r="E2" s="233"/>
+      <c r="B2" s="236"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="86" t="s">

</xml_diff>

<commit_message>
maximum subarray and contains duplicates
</commit_message>
<xml_diff>
--- a/Top300_LeetCode_DSA_Questions.xlsx
+++ b/Top300_LeetCode_DSA_Questions.xlsx
@@ -34,12 +34,12 @@
     <sheet name="Trie" sheetId="20" r:id="rId20"/>
     <sheet name="Greedy" sheetId="21" r:id="rId21"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1411" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1413" uniqueCount="902">
   <si>
     <t>🚀 TOP 300 LeetCode DSA Questions — MNC &amp; Startup Interview Prep</t>
   </si>
@@ -3888,6 +3888,9 @@
     <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3960,9 +3963,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="60" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -4282,22 +4282,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="237" t="s">
+      <c r="A1" s="238" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="235" t="s">
+      <c r="A2" s="236" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="4" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -4657,13 +4657,13 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="238" t="s">
+      <c r="A26" s="239" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="236"/>
-      <c r="C26" s="236"/>
-      <c r="D26" s="236"/>
-      <c r="E26" s="236"/>
+      <c r="B26" s="237"/>
+      <c r="C26" s="237"/>
+      <c r="D26" s="237"/>
+      <c r="E26" s="237"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4690,22 +4690,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="248" t="s">
+      <c r="A1" s="249" t="s">
         <v>414</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>415</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="97" t="s">
@@ -5003,22 +5003,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="249" t="s">
+      <c r="A1" s="250" t="s">
         <v>458</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>459</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="110" t="s">
@@ -5520,22 +5520,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="250" t="s">
+      <c r="A1" s="251" t="s">
         <v>541</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>542</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="123" t="s">
@@ -6003,22 +6003,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="251" t="s">
+      <c r="A1" s="252" t="s">
         <v>618</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>619</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="134" t="s">
@@ -6639,22 +6639,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="252" t="s">
+      <c r="A1" s="253" t="s">
         <v>708</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>709</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="146" t="s">
@@ -6918,22 +6918,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="253" t="s">
+      <c r="A1" s="254" t="s">
         <v>749</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>750</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="157" t="s">
@@ -7180,22 +7180,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="254" t="s">
+      <c r="A1" s="255" t="s">
         <v>775</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>776</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="160" t="s">
@@ -7442,22 +7442,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="255" t="s">
+      <c r="A1" s="256" t="s">
         <v>792</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>793</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="166" t="s">
@@ -7619,22 +7619,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="256" t="s">
+      <c r="A1" s="257" t="s">
         <v>811</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>812</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="169" t="s">
@@ -7881,22 +7881,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="257" t="s">
+      <c r="A1" s="258" t="s">
         <v>846</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>847</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="180" t="s">
@@ -8058,22 +8058,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="241" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -8125,7 +8125,7 @@
       <c r="C5" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="260" t="s">
+      <c r="D5" s="235" t="s">
         <v>80</v>
       </c>
       <c r="E5" s="14" t="s">
@@ -8151,6 +8151,9 @@
       <c r="E6" s="10" t="s">
         <v>84</v>
       </c>
+      <c r="F6" s="233" t="s">
+        <v>901</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
@@ -8159,14 +8162,17 @@
       <c r="B7" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>76</v>
+      <c r="C7" s="15" t="s">
+        <v>107</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>86</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>87</v>
+      </c>
+      <c r="F7" s="233" t="s">
+        <v>901</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8741,22 +8747,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="258" t="s">
+      <c r="A1" s="259" t="s">
         <v>860</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>861</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="190" t="s">
@@ -8850,22 +8856,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="259" t="s">
+      <c r="A1" s="260" t="s">
         <v>871</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>872</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="200" t="s">
@@ -9095,22 +9101,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="241" t="s">
+      <c r="A1" s="242" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>187</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
@@ -9493,22 +9499,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="242" t="s">
+      <c r="A1" s="243" t="s">
         <v>248</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>249</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
@@ -9738,22 +9744,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="244" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>272</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="41" t="s">
@@ -9949,22 +9955,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="244" t="s">
+      <c r="A1" s="245" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>289</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="53" t="s">
@@ -10177,22 +10183,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="245" t="s">
+      <c r="A1" s="246" t="s">
         <v>311</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>312</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="65" t="s">
@@ -10490,22 +10496,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="246" t="s">
+      <c r="A1" s="247" t="s">
         <v>350</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>351</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="77" t="s">
@@ -10667,22 +10673,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="247" t="s">
+      <c r="A1" s="248" t="s">
         <v>370</v>
       </c>
-      <c r="B1" s="236"/>
-      <c r="C1" s="236"/>
-      <c r="D1" s="236"/>
-      <c r="E1" s="236"/>
+      <c r="B1" s="237"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>371</v>
       </c>
-      <c r="B2" s="236"/>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
+      <c r="B2" s="237"/>
+      <c r="C2" s="237"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="86" t="s">

</xml_diff>

<commit_message>
Moving zeros and missing number
</commit_message>
<xml_diff>
--- a/Top300_LeetCode_DSA_Questions.xlsx
+++ b/Top300_LeetCode_DSA_Questions.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1413" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1415" uniqueCount="902">
   <si>
     <t>🚀 TOP 300 LeetCode DSA Questions — MNC &amp; Startup Interview Prep</t>
   </si>
@@ -8191,6 +8191,9 @@
       <c r="E8" s="10" t="s">
         <v>90</v>
       </c>
+      <c r="F8" s="233" t="s">
+        <v>901</v>
+      </c>
     </row>
     <row r="9" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
@@ -8207,6 +8210,9 @@
       </c>
       <c r="E9" s="14" t="s">
         <v>93</v>
+      </c>
+      <c r="F9" s="233" t="s">
+        <v>901</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8729,6 +8735,7 @@
     <hyperlink ref="D5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>